<commit_message>
static snapshot: zero backend, zero CORS, zero ngrok
</commit_message>
<xml_diff>
--- a/Portfolio_Master.xlsx
+++ b/Portfolio_Master.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cards" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sync Log" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Meta" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sync Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5360,7 +5360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7957,6 +7957,60 @@
         </is>
       </c>
       <c r="E96" t="inlineStr">
+        <is>
+          <t>From My Collection CSV - 19.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-04-25T13:38:04.763285</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>csv</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>123698796</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>From My Collection CSV - 19.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-04-25T13:38:04.823692</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>csv</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>111230748</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
         <is>
           <t>From My Collection CSV - 19.csv</t>
         </is>

</xml_diff>